<commit_message>
Tracking xlsx: samakan status dengan ringkasan sebut harga 21 Okt
26 rancangan -> Sebut harga telah dihantar (termasuk Neram 01, Neram 02,
Chalok Barat yang sebelum ini Belum ada permintaan); selebihnya ->
Belum menerima permintaan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tracking FELDA ORDER FARMGUARD 2026.xlsx
+++ b/Tracking FELDA ORDER FARMGUARD 2026.xlsx
@@ -85,7 +85,7 @@
     <t>AIR TAWAR 01</t>
   </si>
   <si>
-    <t>Belum ada permintaan</t>
+    <t>Belum menerima permintaan</t>
   </si>
   <si>
     <t>AIR TAWAR 02</t>
@@ -304,7 +304,7 @@
     <t>JUMLAH</t>
   </si>
   <si>
-    <t>Quotation siap (draf) - belum dihantar</t>
+    <t>Sebut harga telah dihantar</t>
   </si>
   <si>
     <t>Minta harga seunit 4 item (SM Mammoth, Walkie Talkie, Hailer, Blinker). Buat ikut rancangan. | Rujukan: ND/FWSG/Q/2026-10191</t>
@@ -325,7 +325,7 @@
     <t>Minta harga seunit 4 item (SM Mammoth, Walkie Talkie, Hailer, Blinker). Buat ikut rancangan. | Rujukan: ND/FWSG/Q/2026-10196</t>
   </si>
   <si>
-    <t>Quotation NASA DEF siap (draf) - belum dihantar</t>
+    <t>Sebut harga telah dihantar</t>
   </si>
   <si>
     <t>Minta quotation SM Mammoth 2, Blinker 3. Minta 3 vendor. Hantar quotation melalui WhatsApp. | Rujukan: ND/FLSH/Q/2026-10191 (NASA DEF sahaja)</t>
@@ -334,7 +334,7 @@
     <t>Minta quotation ikut screenshot: SM Mammoth 4, Walkie Talkie 2, Hailer 1, Blinker 3. | Rujukan: ND/FBRS/Q/2026-10191</t>
   </si>
   <si>
-    <t>Borang siap diisi (draf) - belum dihantar</t>
+    <t>Sebut harga telah dihantar</t>
   </si>
   <si>
     <t>Minta isi BORANG SEBUT HARGA KIT GAJAH.xls (satu helaian bagi setiap rancangan). | Rujukan: BORANG SEBUT HARGA KIT GAJAH - NASA DEF.xls</t>
@@ -1733,7 +1733,7 @@
       <c r="I30" s="6"/>
       <c r="J30" s="6"/>
       <c r="K30" s="6" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="L30" s="6"/>
     </row>
@@ -1795,7 +1795,7 @@
       <c r="I32" s="6"/>
       <c r="J32" s="6"/>
       <c r="K32" s="6" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="L32" s="6"/>
     </row>
@@ -1823,7 +1823,7 @@
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
       <c r="K33" s="6" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="L33" s="6"/>
     </row>

</xml_diff>

<commit_message>
Tenggaroh Selatan 01: sebut harga dihantar (RM7,450); sync contact & catatan dengan Excel
- data.js: Tenggaroh Selatan 01 -> Requested, ND/FWJB/Q/2026-10211, En. Badrul
- data.js: contact, tel, alamat & catatan disegerakkan dengan Excel tracking (Jengka: penyelaras setiap rancangan)
- app.js: jumlah RM sebut harga dipapar dalam ringkasan sidebar (ikut penapis)
- PLANNING.md: 15 pending / 27 requested, jumlah RM 249,365

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tracking FELDA ORDER FARMGUARD 2026.xlsx
+++ b/Tracking FELDA ORDER FARMGUARD 2026.xlsx
@@ -5,37 +5,29 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\IzwanSYSTEC\NASA DEF\Projek Gajah - Farmguard\Felda - HQ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\NASA DEF\Projek Gajah - Farmguard\Felda - HQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203E70DC-D9E9-478E-83FA-CDB2AA307E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9FDFDB4-DFA4-439C-85F0-8FD0AEF10B3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28440" yWindow="-984" windowWidth="20640" windowHeight="14328" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracking" sheetId="1" r:id="rId1"/>
+    <sheet name="Tracking (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tracking!$A$4:$L$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tracking!$A$4:$L$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tracking (2)'!$A$4:$L$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Tracking!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Tracking (2)'!$4:$4</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="150">
   <si>
     <t>TRACKING PEMBEKALAN KIT GAJAH FELDA 2026</t>
   </si>
@@ -85,7 +77,7 @@
     <t>AIR TAWAR 01</t>
   </si>
   <si>
-    <t>Belum menerima permintaan</t>
+    <t>Belum ada permintaan</t>
   </si>
   <si>
     <t>AIR TAWAR 02</t>
@@ -304,7 +296,7 @@
     <t>JUMLAH</t>
   </si>
   <si>
-    <t>Sebut harga telah dihantar</t>
+    <t>Quotation siap (draf) - belum dihantar</t>
   </si>
   <si>
     <t>Minta harga seunit 4 item (SM Mammoth, Walkie Talkie, Hailer, Blinker). Buat ikut rancangan. | Rujukan: ND/FWSG/Q/2026-10191</t>
@@ -325,7 +317,7 @@
     <t>Minta harga seunit 4 item (SM Mammoth, Walkie Talkie, Hailer, Blinker). Buat ikut rancangan. | Rujukan: ND/FWSG/Q/2026-10196</t>
   </si>
   <si>
-    <t>Sebut harga telah dihantar</t>
+    <t>Quotation NASA DEF siap (draf) - belum dihantar</t>
   </si>
   <si>
     <t>Minta quotation SM Mammoth 2, Blinker 3. Minta 3 vendor. Hantar quotation melalui WhatsApp. | Rujukan: ND/FLSH/Q/2026-10191 (NASA DEF sahaja)</t>
@@ -334,7 +326,7 @@
     <t>Minta quotation ikut screenshot: SM Mammoth 4, Walkie Talkie 2, Hailer 1, Blinker 3. | Rujukan: ND/FBRS/Q/2026-10191</t>
   </si>
   <si>
-    <t>Sebut harga telah dihantar</t>
+    <t>Borang siap diisi (draf) - belum dihantar</t>
   </si>
   <si>
     <t>Minta isi BORANG SEBUT HARGA KIT GAJAH.xls (satu helaian bagi setiap rancangan). | Rujukan: BORANG SEBUT HARGA KIT GAJAH - NASA DEF.xls</t>
@@ -343,15 +335,6 @@
     <t>Bertanya tentang SM Mammoth. Beri quotation sahaja. | Rujukan: ND/FCRL/Q/2026-10191</t>
   </si>
   <si>
-    <t>Minta quotation ikut rancangan, SM Mammoth/FarmGuard sahaja (2 unit), untuk permohonan aset. Delivery RM50/unit. Quotation gabungan (1 unit) dah dibuat 18/10/2026. | Rujukan: ND/FWGM/Q/2026-10191</t>
-  </si>
-  <si>
-    <t>Minta quotation ikut rancangan, SM Mammoth/FarmGuard sahaja (2 unit), untuk permohonan aset. Delivery RM50/unit. Quotation gabungan (1 unit) dah dibuat 18/10/2026. | Rujukan: ND/FWGM/Q/2026-10192</t>
-  </si>
-  <si>
-    <t>Minta quotation ikut rancangan, SM Mammoth/FarmGuard sahaja (2 unit), untuk permohonan aset. Delivery RM50/unit. Quotation gabungan (1 unit) dah dibuat 18/10/2026. | Rujukan: ND/FWGM/Q/2026-10193</t>
-  </si>
-  <si>
     <t>Minta sebut harga SM Mammoth/FarmGuard sahaja dulu, untuk permohonan no. aset peringkat HQ. | Rujukan: ND/FWJK/Q/2026-10191</t>
   </si>
   <si>
@@ -364,7 +347,137 @@
     <t>Minta sebut harga SM Mammoth/FarmGuard sahaja dulu, untuk permohonan no. aset peringkat HQ. | Rujukan: ND/FWJK/Q/2026-10194</t>
   </si>
   <si>
+    <t>Quotation R1 siap - belum dihantar</t>
+  </si>
+  <si>
+    <t>Minta quotation ikut rancangan, SM Mammoth/FarmGuard sahaja (2 unit), untuk permohonan aset. Delivery RM50/unit. Quotation gabungan (1 unit) dah dibuat 18/10/2026. | Rujukan: ND/FWGM/Q/2026-10191 | R1 (21/10/2026): ND/FWGM/Q/2026-10191R1 - semua produk, FarmGuard RM2,900 termasuk delivery + training, TOTAL RM7,045</t>
+  </si>
+  <si>
+    <t>Minta quotation ikut rancangan, SM Mammoth/FarmGuard sahaja (2 unit), untuk permohonan aset. Delivery RM50/unit. Quotation gabungan (1 unit) dah dibuat 18/10/2026. | Rujukan: ND/FWGM/Q/2026-10192 | R1 (21/10/2026): ND/FWGM/Q/2026-10192R1 - semua produk, FarmGuard RM2,900 termasuk delivery + training, TOTAL RM7,045</t>
+  </si>
+  <si>
+    <t>Minta quotation ikut rancangan, SM Mammoth/FarmGuard sahaja (2 unit), untuk permohonan aset. Delivery RM50/unit. Quotation gabungan (1 unit) dah dibuat 18/10/2026. | Rujukan: ND/FWGM/Q/2026-10193 | R1 (21/10/2026): ND/FWGM/Q/2026-10193R1 - semua produk, FarmGuard RM2,900 termasuk delivery + training, TOTAL RM7,045</t>
+  </si>
+  <si>
     <t>NITAR 01</t>
+  </si>
+  <si>
+    <t>Sudah dihantar</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWSG/Q/2026-10191R1 (RM12,845) | Minta harga seunit 4 item (SM Mammoth, Walkie Talkie, Hailer, Blinker). Buat ikut rancangan. | Rujukan: ND/FWSG/Q/2026-10191</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWSG/Q/2026-10192R1 (RM9,945) | Minta harga seunit 4 item (SM Mammoth, Walkie Talkie, Hailer, Blinker). Buat ikut rancangan. | Rujukan: ND/FWSG/Q/2026-10192</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWSG/Q/2026-10193R1 (RM9,945) | Minta harga seunit 4 item (SM Mammoth, Walkie Talkie, Hailer, Blinker). Buat ikut rancangan. | Rujukan: ND/FWSG/Q/2026-10193</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWSG/Q/2026-10194R1 (RM8,850) | Minta harga seunit 4 item (SM Mammoth, Walkie Talkie, Hailer, Blinker). Buat ikut rancangan. | Rujukan: ND/FWSG/Q/2026-10194</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWSG/Q/2026-10195R1 (RM9,945) | Minta harga seunit 4 item (SM Mammoth, Walkie Talkie, Hailer, Blinker). Buat ikut rancangan. | Rujukan: ND/FWSG/Q/2026-10195</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWSG/Q/2026-10196R1 (RM7,045) | Minta harga seunit 4 item (SM Mammoth, Walkie Talkie, Hailer, Blinker). Buat ikut rancangan. | Rujukan: ND/FWSG/Q/2026-10196</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FLSH/Q/2026-10191 (RM5,950) + Surat Pembekal Tunggal ND/S/FLSH/2026-10201 | Minta quotation SM Mammoth 2, Blinker 3. Minta 3 vendor. Hantar quotation melalui WhatsApp. | Rujukan: ND/FLSH/Q/2026-10191 (NASA DEF sahaja)</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FBRS/Q/2026-10191 (RM12,845) | Minta quotation ikut screenshot: SM Mammoth 4, Walkie Talkie 2, Hailer 1, Blinker 3. | Rujukan: ND/FBRS/Q/2026-10191</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: Borang Sebut Harga Kit Gajah - NASA DEF R1, helaian BS1 (RM11,750) | Minta isi BORANG SEBUT HARGA KIT GAJAH.xls (satu helaian bagi setiap rancangan). | Rujukan: BORANG SEBUT HARGA KIT GAJAH - NASA DEF.xls</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: Borang Sebut Harga Kit Gajah - NASA DEF R1, helaian BS23 (RM12,845) | Minta isi BORANG SEBUT HARGA KIT GAJAH.xls (satu helaian bagi setiap rancangan). | Rujukan: BORANG SEBUT HARGA KIT GAJAH - NASA DEF.xls</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: Borang Sebut Harga Kit Gajah - NASA DEF R1, helaian BK (RM5,950) | Minta isi BORANG SEBUT HARGA KIT GAJAH.xls (satu helaian bagi setiap rancangan). | Rujukan: BORANG SEBUT HARGA KIT GAJAH - NASA DEF.xls</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: Borang Sebut Harga Kit Gajah - NASA DEF R1, helaian LU1 (RM9,945) | Minta isi BORANG SEBUT HARGA KIT GAJAH.xls (satu helaian bagi setiap rancangan). | Rujukan: BORANG SEBUT HARGA KIT GAJAH - NASA DEF.xls</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: Borang Sebut Harga Kit Gajah - NASA DEF R1, helaian LU24 (RM9,945) | Minta isi BORANG SEBUT HARGA KIT GAJAH.xls (satu helaian bagi setiap rancangan). | Rujukan: BORANG SEBUT HARGA KIT GAJAH - NASA DEF.xls</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: Borang Sebut Harga Kit Gajah - NASA DEF R1, helaian SPU (RM7,045) | Minta isi BORANG SEBUT HARGA KIT GAJAH.xls (satu helaian bagi setiap rancangan). | Rujukan: BORANG SEBUT HARGA KIT GAJAH - NASA DEF.xls</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: Borang Sebut Harga Kit Gajah - NASA DEF R1, helaian SPS (RM7,045) | Minta isi BORANG SEBUT HARGA KIT GAJAH.xls (satu helaian bagi setiap rancangan). | Rujukan: BORANG SEBUT HARGA KIT GAJAH - NASA DEF.xls</t>
+  </si>
+  <si>
+    <t>Pejabat FELDA Wilayah Terengganu, Lot 10260, Tepoh, Mukim Kuala Nerus, 21060 Kuala Terengganu</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWTG/Q/2026-10211 (RM9,945)</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWTG/Q/2026-10212 (RM11,750); terdahulu ND/FCRL/Q/2026-10191 | Bertanya tentang SM Mammoth. Beri quotation sahaja. | Rujukan: ND/FCRL/Q/2026-10191</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWTG/Q/2026-10213 (RM9,945)</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWTG/Q/2026-10214 (RM7,045)</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWGM/Q/2026-10191R1 (RM7,045) | Minta quotation ikut rancangan, SM Mammoth/FarmGuard sahaja (2 unit), untuk permohonan aset. Delivery RM50/unit. Quotation gabungan (1 unit) dah dibuat 18/10/2026. | Rujukan: ND/FWGM/Q/2026-10191 | R1 (21/10/2026): ND/FWGM/Q/2026-10191R1 - semua produk, FarmGuard RM2,900 termasuk delivery + training, TOTAL RM7,045</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWGM/Q/2026-10192R1 (RM7,045) | Minta quotation ikut rancangan, SM Mammoth/FarmGuard sahaja (2 unit), untuk permohonan aset. Delivery RM50/unit. Quotation gabungan (1 unit) dah dibuat 18/10/2026. | Rujukan: ND/FWGM/Q/2026-10192 | R1 (21/10/2026): ND/FWGM/Q/2026-10192R1 - semua produk, FarmGuard RM2,900 termasuk delivery + training, TOTAL RM7,045</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWGM/Q/2026-10193R1 (RM7,045) | Minta quotation ikut rancangan, SM Mammoth/FarmGuard sahaja (2 unit), untuk permohonan aset. Delivery RM50/unit. Quotation gabungan (1 unit) dah dibuat 18/10/2026. | Rujukan: ND/FWGM/Q/2026-10193 | R1 (21/10/2026): ND/FWGM/Q/2026-10193R1 - semua produk, FarmGuard RM2,900 termasuk delivery + training, TOTAL RM7,045</t>
+  </si>
+  <si>
+    <t>Nasrullah (Penyelaras Kit Gajah)</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWJK/Q/2026-10191R1 (RM10,450) | Minta sebut harga SM Mammoth/FarmGuard sahaja dulu, untuk permohonan no. aset peringkat HQ. | Rujukan: ND/FWJK/Q/2026-10191</t>
+  </si>
+  <si>
+    <t>Azwani (Penyelaras Kit Gajah)</t>
+  </si>
+  <si>
+    <t>+60 11-5198 3566</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWJK/Q/2026-10192R1 (RM10,150) + ND/FKG4/Q/2026-10191 (Kerani, RM9,700) | Kerani minta quotation: SM Mammoth 3, Walkie Talkie 2, Blinker 3. Termasuk juga dalam permintaan Wilayah Jengka (Nashrul, +60 14-826 8464): Minta sebut harga SM Mammoth/FarmGuard sahaja dulu, untuk permohonan no. aset peringkat HQ. | Rujukan: ND/FWJK/Q/2026-10192 (Wilayah, FarmGuard sahaja) + ND/FKG4/Q/2026-10191 (Kerani KG4)</t>
+  </si>
+  <si>
+    <t>Ruzaini (Penyelaras Kit Gajah)</t>
+  </si>
+  <si>
+    <t>+60 19-661 8691</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWJK/Q/2026-10193R1 (RM9,450) | Minta sebut harga SM Mammoth/FarmGuard sahaja dulu, untuk permohonan no. aset peringkat HQ. | Rujukan: ND/FWJK/Q/2026-10193</t>
+  </si>
+  <si>
+    <t>Nizam (Penyelaras Kit Gajah)</t>
+  </si>
+  <si>
+    <t>+60 11-2904 2423</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWJK/Q/2026-10194R1 (RM10,150) | Minta sebut harga SM Mammoth/FarmGuard sahaja dulu, untuk permohonan no. aset peringkat HQ. | Rujukan: ND/FWJK/Q/2026-10194</t>
+  </si>
+  <si>
+    <t>En.badrul +60 19-910 0609 Rancangan Tenggaroh 1</t>
+  </si>
+  <si>
+    <t>Telefon: 07-236 1477 / 07-236 1478</t>
+  </si>
+  <si>
+    <t>Jalan Taruka, Off Jalan Datin Halimah, Karung Berkunci 724, 
+80990 Johor Bahru, Johor Darul Takzim.</t>
+  </si>
+  <si>
+    <t>Versi terkini dihantar: ND/FWJB/Q/2026-10211 (RM7,450) | En. Badrul minta: SM Mammoth 2 unit (bekal dan pasang), Walkie Talkie 2, Hailer 1, Blinker 3. Harga: FarmGuard RM3,000 (termasuk bekal &amp; pasang), Walkie Talkie RM500, Hailer RM300, Blinker RM50. | Rujukan: ND/FWJB/Q/2026-10211</t>
   </si>
 </sst>
 </file>
@@ -409,7 +522,7 @@
       <name val="Segoe UI"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -434,6 +547,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEEF5F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCEEED4"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -488,7 +607,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -510,11 +629,19 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -820,7 +947,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -884,8 +1011,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+    <row r="5" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="5">
@@ -914,8 +1041,8 @@
       </c>
       <c r="L5" s="6"/>
     </row>
-    <row r="6" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10"/>
+    <row r="6" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13"/>
       <c r="B6" s="5">
         <v>2</v>
       </c>
@@ -942,8 +1069,8 @@
       </c>
       <c r="L6" s="6"/>
     </row>
-    <row r="7" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10"/>
+    <row r="7" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13"/>
       <c r="B7" s="5">
         <v>3</v>
       </c>
@@ -970,8 +1097,8 @@
       </c>
       <c r="L7" s="6"/>
     </row>
-    <row r="8" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
+    <row r="8" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13"/>
       <c r="B8" s="5">
         <v>4</v>
       </c>
@@ -998,8 +1125,8 @@
       </c>
       <c r="L8" s="6"/>
     </row>
-    <row r="9" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
+    <row r="9" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="13"/>
       <c r="B9" s="5">
         <v>5</v>
       </c>
@@ -1026,8 +1153,8 @@
       </c>
       <c r="L9" s="6"/>
     </row>
-    <row r="10" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
+    <row r="10" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13"/>
       <c r="B10" s="5">
         <v>6</v>
       </c>
@@ -1054,8 +1181,8 @@
       </c>
       <c r="L10" s="6"/>
     </row>
-    <row r="11" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
+    <row r="11" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13"/>
       <c r="B11" s="5">
         <v>7</v>
       </c>
@@ -1082,8 +1209,8 @@
       </c>
       <c r="L11" s="6"/>
     </row>
-    <row r="12" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
+    <row r="12" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13"/>
       <c r="B12" s="5">
         <v>8</v>
       </c>
@@ -1110,8 +1237,8 @@
       </c>
       <c r="L12" s="6"/>
     </row>
-    <row r="13" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10"/>
+    <row r="13" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13"/>
       <c r="B13" s="5">
         <v>9</v>
       </c>
@@ -1138,8 +1265,8 @@
       </c>
       <c r="L13" s="6"/>
     </row>
-    <row r="14" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
+    <row r="14" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="14"/>
       <c r="B14" s="5">
         <v>10</v>
       </c>
@@ -1158,6 +1285,1424 @@
       <c r="G14" s="5">
         <v>3</v>
       </c>
+      <c r="H14" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="I14" s="6"/>
+      <c r="J14" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="5">
+        <v>11</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" s="5">
+        <v>3</v>
+      </c>
+      <c r="E15" s="5">
+        <v>2</v>
+      </c>
+      <c r="F15" s="5">
+        <v>1</v>
+      </c>
+      <c r="G15" s="5">
+        <v>3</v>
+      </c>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+    </row>
+    <row r="16" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="5">
+        <v>12</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="5">
+        <v>4</v>
+      </c>
+      <c r="E16" s="5">
+        <v>2</v>
+      </c>
+      <c r="F16" s="5">
+        <v>1</v>
+      </c>
+      <c r="G16" s="5">
+        <v>3</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13"/>
+      <c r="B17" s="5">
+        <v>13</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="5">
+        <v>3</v>
+      </c>
+      <c r="E17" s="5">
+        <v>2</v>
+      </c>
+      <c r="F17" s="5">
+        <v>1</v>
+      </c>
+      <c r="G17" s="5">
+        <v>3</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J17" t="s">
+        <v>147</v>
+      </c>
+      <c r="K17" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="13"/>
+      <c r="B18" s="5">
+        <v>14</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="5">
+        <v>3</v>
+      </c>
+      <c r="E18" s="5">
+        <v>2</v>
+      </c>
+      <c r="F18" s="5">
+        <v>1</v>
+      </c>
+      <c r="G18" s="5">
+        <v>3</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="13"/>
+      <c r="B19" s="5">
+        <v>15</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="5">
+        <v>3</v>
+      </c>
+      <c r="E19" s="5">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5">
+        <v>3</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="13"/>
+      <c r="B20" s="5">
+        <v>16</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="5">
+        <v>3</v>
+      </c>
+      <c r="E20" s="5">
+        <v>2</v>
+      </c>
+      <c r="F20" s="5">
+        <v>1</v>
+      </c>
+      <c r="G20" s="5">
+        <v>3</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K20" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="14"/>
+      <c r="B21" s="5">
+        <v>17</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" s="5">
+        <v>2</v>
+      </c>
+      <c r="E21" s="5">
+        <v>2</v>
+      </c>
+      <c r="F21" s="5">
+        <v>1</v>
+      </c>
+      <c r="G21" s="5">
+        <v>3</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="5">
+        <v>18</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="5">
+        <v>2</v>
+      </c>
+      <c r="E22" s="5">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5">
+        <v>3</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="J22" s="6"/>
+      <c r="K22" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="14"/>
+      <c r="B23" s="5">
+        <v>19</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="5">
+        <v>4</v>
+      </c>
+      <c r="E23" s="5">
+        <v>2</v>
+      </c>
+      <c r="F23" s="5">
+        <v>1</v>
+      </c>
+      <c r="G23" s="5">
+        <v>3</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K23" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" s="5">
+        <v>20</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" s="5">
+        <v>4</v>
+      </c>
+      <c r="E24" s="5">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5">
+        <v>3</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K24" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="13"/>
+      <c r="B25" s="5">
+        <v>21</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D25" s="5">
+        <v>4</v>
+      </c>
+      <c r="E25" s="5">
+        <v>2</v>
+      </c>
+      <c r="F25" s="5">
+        <v>1</v>
+      </c>
+      <c r="G25" s="5">
+        <v>3</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K25" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="13"/>
+      <c r="B26" s="5">
+        <v>22</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" s="5">
+        <v>2</v>
+      </c>
+      <c r="E26" s="5">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5">
+        <v>0</v>
+      </c>
+      <c r="G26" s="5">
+        <v>3</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K26" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="13"/>
+      <c r="B27" s="5">
+        <v>23</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" s="5">
+        <v>3</v>
+      </c>
+      <c r="E27" s="5">
+        <v>2</v>
+      </c>
+      <c r="F27" s="5">
+        <v>1</v>
+      </c>
+      <c r="G27" s="5">
+        <v>3</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K27" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="13"/>
+      <c r="B28" s="5">
+        <v>24</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D28" s="5">
+        <v>3</v>
+      </c>
+      <c r="E28" s="5">
+        <v>2</v>
+      </c>
+      <c r="F28" s="5">
+        <v>1</v>
+      </c>
+      <c r="G28" s="5">
+        <v>3</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K28" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="13"/>
+      <c r="B29" s="5">
+        <v>25</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D29" s="5">
+        <v>2</v>
+      </c>
+      <c r="E29" s="5">
+        <v>2</v>
+      </c>
+      <c r="F29" s="5">
+        <v>1</v>
+      </c>
+      <c r="G29" s="5">
+        <v>3</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K29" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="14"/>
+      <c r="B30" s="5">
+        <v>26</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D30" s="5">
+        <v>2</v>
+      </c>
+      <c r="E30" s="5">
+        <v>2</v>
+      </c>
+      <c r="F30" s="5">
+        <v>1</v>
+      </c>
+      <c r="G30" s="5">
+        <v>3</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L30" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" s="5">
+        <v>27</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D31" s="5">
+        <v>3</v>
+      </c>
+      <c r="E31" s="5">
+        <v>2</v>
+      </c>
+      <c r="F31" s="5">
+        <v>1</v>
+      </c>
+      <c r="G31" s="5">
+        <v>3</v>
+      </c>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="K31" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="13"/>
+      <c r="B32" s="5">
+        <v>28</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D32" s="5">
+        <v>4</v>
+      </c>
+      <c r="E32" s="5">
+        <v>0</v>
+      </c>
+      <c r="F32" s="5">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5">
+        <v>3</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="K32" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="13"/>
+      <c r="B33" s="5">
+        <v>29</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D33" s="5">
+        <v>3</v>
+      </c>
+      <c r="E33" s="5">
+        <v>2</v>
+      </c>
+      <c r="F33" s="5">
+        <v>1</v>
+      </c>
+      <c r="G33" s="5">
+        <v>3</v>
+      </c>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="14"/>
+      <c r="B34" s="5">
+        <v>30</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D34" s="5">
+        <v>2</v>
+      </c>
+      <c r="E34" s="5">
+        <v>2</v>
+      </c>
+      <c r="F34" s="5">
+        <v>1</v>
+      </c>
+      <c r="G34" s="5">
+        <v>3</v>
+      </c>
+      <c r="H34" s="6"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="K34" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="5">
+        <v>31</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D35" s="5">
+        <v>2</v>
+      </c>
+      <c r="E35" s="5">
+        <v>2</v>
+      </c>
+      <c r="F35" s="5">
+        <v>1</v>
+      </c>
+      <c r="G35" s="5">
+        <v>3</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="K35" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="13"/>
+      <c r="B36" s="5">
+        <v>32</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D36" s="5">
+        <v>2</v>
+      </c>
+      <c r="E36" s="5">
+        <v>2</v>
+      </c>
+      <c r="F36" s="5">
+        <v>1</v>
+      </c>
+      <c r="G36" s="5">
+        <v>3</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K36" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="14"/>
+      <c r="B37" s="5">
+        <v>33</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D37" s="5">
+        <v>2</v>
+      </c>
+      <c r="E37" s="5">
+        <v>2</v>
+      </c>
+      <c r="F37" s="5">
+        <v>1</v>
+      </c>
+      <c r="G37" s="5">
+        <v>3</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="K37" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B38" s="5">
+        <v>34</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D38" s="5">
+        <v>3</v>
+      </c>
+      <c r="E38" s="5">
+        <v>2</v>
+      </c>
+      <c r="F38" s="5">
+        <v>1</v>
+      </c>
+      <c r="G38" s="5">
+        <v>3</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="J38" s="6"/>
+      <c r="K38" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="87" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="13"/>
+      <c r="B39" s="5">
+        <v>35</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="D39" s="5">
+        <v>3</v>
+      </c>
+      <c r="E39" s="5">
+        <v>2</v>
+      </c>
+      <c r="F39" s="5">
+        <v>0</v>
+      </c>
+      <c r="G39" s="5">
+        <v>3</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="K39" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="13"/>
+      <c r="B40" s="5">
+        <v>36</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D40" s="5">
+        <v>3</v>
+      </c>
+      <c r="E40" s="5">
+        <v>0</v>
+      </c>
+      <c r="F40" s="5">
+        <v>1</v>
+      </c>
+      <c r="G40" s="5">
+        <v>3</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="J40" s="6"/>
+      <c r="K40" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="14"/>
+      <c r="B41" s="5">
+        <v>37</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D41" s="5">
+        <v>3</v>
+      </c>
+      <c r="E41" s="5">
+        <v>2</v>
+      </c>
+      <c r="F41" s="5">
+        <v>0</v>
+      </c>
+      <c r="G41" s="5">
+        <v>3</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="J41" s="6"/>
+      <c r="K41" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L41" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B42" s="5">
+        <v>38</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D42" s="5">
+        <v>0</v>
+      </c>
+      <c r="E42" s="5">
+        <v>0</v>
+      </c>
+      <c r="F42" s="5">
+        <v>0</v>
+      </c>
+      <c r="G42" s="5">
+        <v>3</v>
+      </c>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="6"/>
+      <c r="K42" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L42" s="6"/>
+    </row>
+    <row r="43" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="13"/>
+      <c r="B43" s="5">
+        <v>39</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D43" s="5">
+        <v>0</v>
+      </c>
+      <c r="E43" s="5">
+        <v>2</v>
+      </c>
+      <c r="F43" s="5">
+        <v>1</v>
+      </c>
+      <c r="G43" s="5">
+        <v>3</v>
+      </c>
+      <c r="H43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="6"/>
+      <c r="K43" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L43" s="6"/>
+    </row>
+    <row r="44" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="13"/>
+      <c r="B44" s="5">
+        <v>40</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D44" s="5">
+        <v>0</v>
+      </c>
+      <c r="E44" s="5">
+        <v>0</v>
+      </c>
+      <c r="F44" s="5">
+        <v>0</v>
+      </c>
+      <c r="G44" s="5">
+        <v>3</v>
+      </c>
+      <c r="H44" s="6"/>
+      <c r="I44" s="6"/>
+      <c r="J44" s="6"/>
+      <c r="K44" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L44" s="6"/>
+    </row>
+    <row r="45" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="13"/>
+      <c r="B45" s="5">
+        <v>41</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D45" s="5">
+        <v>2</v>
+      </c>
+      <c r="E45" s="5">
+        <v>0</v>
+      </c>
+      <c r="F45" s="5">
+        <v>0</v>
+      </c>
+      <c r="G45" s="5">
+        <v>3</v>
+      </c>
+      <c r="H45" s="6"/>
+      <c r="I45" s="6"/>
+      <c r="J45" s="6"/>
+      <c r="K45" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L45" s="6"/>
+    </row>
+    <row r="46" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="13"/>
+      <c r="B46" s="5">
+        <v>42</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D46" s="5">
+        <v>2</v>
+      </c>
+      <c r="E46" s="5">
+        <v>2</v>
+      </c>
+      <c r="F46" s="5">
+        <v>1</v>
+      </c>
+      <c r="G46" s="5">
+        <v>3</v>
+      </c>
+      <c r="H46" s="6"/>
+      <c r="I46" s="6"/>
+      <c r="J46" s="6"/>
+      <c r="K46" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L46" s="6"/>
+    </row>
+    <row r="47" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="14"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="D47" s="8">
+        <f>SUM(D5:D46)</f>
+        <v>97</v>
+      </c>
+      <c r="E47" s="8">
+        <f>SUM(E5:E46)</f>
+        <v>62</v>
+      </c>
+      <c r="F47" s="8">
+        <f>SUM(F5:F46)</f>
+        <v>31</v>
+      </c>
+      <c r="G47" s="8">
+        <f>SUM(G5:G46)</f>
+        <v>126</v>
+      </c>
+      <c r="H47" s="8"/>
+      <c r="I47" s="8"/>
+      <c r="J47" s="8"/>
+      <c r="K47" s="8"/>
+      <c r="L47" s="8"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A48" s="8"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:L47" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <mergeCells count="8">
+    <mergeCell ref="A5:A14"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A42:A47"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="A16:A21"/>
+    <mergeCell ref="A24:A30"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A38:A41"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D2BF3F4-3D94-46A4-8D85-3721B780CAD3}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L53"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="6" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="7" width="9" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="10" max="10" width="44" customWidth="1"/>
+    <col min="11" max="11" width="30" customWidth="1"/>
+    <col min="12" max="12" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="18.75" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" s="6"/>
+    </row>
+    <row r="6" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13"/>
+      <c r="B6" s="5">
+        <v>2</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L6" s="6"/>
+    </row>
+    <row r="7" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13"/>
+      <c r="B7" s="5">
+        <v>3</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L7" s="6"/>
+    </row>
+    <row r="8" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13"/>
+      <c r="B8" s="5">
+        <v>4</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L8" s="6"/>
+    </row>
+    <row r="9" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="13"/>
+      <c r="B9" s="5">
+        <v>5</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L9" s="6"/>
+    </row>
+    <row r="10" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13"/>
+      <c r="B10" s="5">
+        <v>6</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="6"/>
+    </row>
+    <row r="11" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13"/>
+      <c r="B11" s="5">
+        <v>7</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L11" s="6"/>
+    </row>
+    <row r="12" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13"/>
+      <c r="B12" s="5">
+        <v>8</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L12" s="6"/>
+    </row>
+    <row r="13" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13"/>
+      <c r="B13" s="5">
+        <v>9</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L13" s="6"/>
+    </row>
+    <row r="14" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="14"/>
+      <c r="B14" s="5">
+        <v>10</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
@@ -1167,39 +2712,29 @@
       <c r="L14" s="6"/>
     </row>
     <row r="15" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>26</v>
-      </c>
+      <c r="A15" s="9"/>
       <c r="B15" s="5">
         <v>11</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="D15" s="5">
-        <v>3</v>
-      </c>
-      <c r="E15" s="5">
-        <v>2</v>
-      </c>
-      <c r="F15" s="5">
-        <v>1</v>
-      </c>
-      <c r="G15" s="5">
-        <v>3</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
       <c r="J15" s="6"/>
-      <c r="K15" s="6" t="s">
-        <v>16</v>
-      </c>
+      <c r="K15" s="6"/>
       <c r="L15" s="6"/>
     </row>
     <row r="16" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
+      <c r="A16" s="12" t="s">
+        <v>26</v>
+      </c>
       <c r="B16" s="5">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>27</v>
@@ -1233,9 +2768,9 @@
       </c>
     </row>
     <row r="17" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10"/>
+      <c r="A17" s="13"/>
       <c r="B17" s="5">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>31</v>
@@ -1269,9 +2804,9 @@
       </c>
     </row>
     <row r="18" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
+      <c r="A18" s="13"/>
       <c r="B18" s="5">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>32</v>
@@ -1305,9 +2840,9 @@
       </c>
     </row>
     <row r="19" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10"/>
+      <c r="A19" s="13"/>
       <c r="B19" s="5">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>33</v>
@@ -1341,9 +2876,9 @@
       </c>
     </row>
     <row r="20" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
+      <c r="A20" s="13"/>
       <c r="B20" s="5">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>34</v>
@@ -1377,9 +2912,9 @@
       </c>
     </row>
     <row r="21" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="11"/>
+      <c r="A21" s="14"/>
       <c r="B21" s="5">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>35</v>
@@ -1413,11 +2948,11 @@
       </c>
     </row>
     <row r="22" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="12" t="s">
         <v>36</v>
       </c>
       <c r="B22" s="5">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>37</v>
@@ -1449,9 +2984,9 @@
       </c>
     </row>
     <row r="23" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="11"/>
+      <c r="A23" s="14"/>
       <c r="B23" s="5">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>40</v>
@@ -1485,11 +3020,11 @@
       </c>
     </row>
     <row r="24" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B24" s="5">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>45</v>
@@ -1523,9 +3058,9 @@
       </c>
     </row>
     <row r="25" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10"/>
+      <c r="A25" s="13"/>
       <c r="B25" s="5">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>49</v>
@@ -1559,9 +3094,9 @@
       </c>
     </row>
     <row r="26" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10"/>
+      <c r="A26" s="13"/>
       <c r="B26" s="5">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>50</v>
@@ -1595,9 +3130,9 @@
       </c>
     </row>
     <row r="27" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="10"/>
+      <c r="A27" s="13"/>
       <c r="B27" s="5">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>51</v>
@@ -1631,9 +3166,9 @@
       </c>
     </row>
     <row r="28" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10"/>
+      <c r="A28" s="13"/>
       <c r="B28" s="5">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>52</v>
@@ -1667,9 +3202,9 @@
       </c>
     </row>
     <row r="29" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="10"/>
+      <c r="A29" s="13"/>
       <c r="B29" s="5">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>53</v>
@@ -1703,9 +3238,9 @@
       </c>
     </row>
     <row r="30" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="11"/>
+      <c r="A30" s="14"/>
       <c r="B30" s="5">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>54</v>
@@ -1739,39 +3274,31 @@
       </c>
     </row>
     <row r="31" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="12" t="s">
         <v>55</v>
       </c>
       <c r="B31" s="5">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D31" s="5">
-        <v>3</v>
-      </c>
-      <c r="E31" s="5">
-        <v>2</v>
-      </c>
-      <c r="F31" s="5">
-        <v>1</v>
-      </c>
-      <c r="G31" s="5">
-        <v>3</v>
-      </c>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
       <c r="H31" s="6"/>
       <c r="I31" s="6"/>
       <c r="J31" s="6"/>
       <c r="K31" s="6" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="L31" s="6"/>
     </row>
     <row r="32" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="10"/>
+      <c r="A32" s="13"/>
       <c r="B32" s="5">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>57</v>
@@ -1803,67 +3330,51 @@
       </c>
     </row>
     <row r="33" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="10"/>
+      <c r="A33" s="13"/>
       <c r="B33" s="5">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D33" s="5">
-        <v>3</v>
-      </c>
-      <c r="E33" s="5">
-        <v>2</v>
-      </c>
-      <c r="F33" s="5">
-        <v>1</v>
-      </c>
-      <c r="G33" s="5">
-        <v>3</v>
-      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
       <c r="H33" s="6"/>
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
       <c r="K33" s="6" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="L33" s="6"/>
     </row>
     <row r="34" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="11"/>
+      <c r="A34" s="14"/>
       <c r="B34" s="5">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D34" s="5">
-        <v>2</v>
-      </c>
-      <c r="E34" s="5">
-        <v>2</v>
-      </c>
-      <c r="F34" s="5">
-        <v>1</v>
-      </c>
-      <c r="G34" s="5">
-        <v>3</v>
-      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
       <c r="K34" s="6" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="L34" s="6"/>
     </row>
-    <row r="35" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="9" t="s">
+    <row r="35" spans="1:12" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
         <v>62</v>
       </c>
       <c r="B35" s="5">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>63</v>
@@ -1890,16 +3401,16 @@
         <v>66</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="10"/>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="13"/>
       <c r="B36" s="5">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>67</v>
@@ -1926,16 +3437,16 @@
         <v>68</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="11"/>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="14"/>
       <c r="B37" s="5">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>69</v>
@@ -1962,18 +3473,18 @@
         <v>70</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
+      <c r="A38" s="12" t="s">
         <v>71</v>
       </c>
       <c r="B38" s="5">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>72</v>
@@ -2001,13 +3512,13 @@
         <v>89</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="39" spans="1:12" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="10"/>
+      <c r="A39" s="13"/>
       <c r="B39" s="5">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>75</v>
@@ -2037,13 +3548,13 @@
         <v>89</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="40" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="10"/>
+      <c r="A40" s="13"/>
       <c r="B40" s="5">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>79</v>
@@ -2071,13 +3582,13 @@
         <v>89</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="11"/>
+      <c r="A41" s="14"/>
       <c r="B41" s="5">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>80</v>
@@ -2105,31 +3616,23 @@
         <v>89</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="9" t="s">
+      <c r="A42" s="12" t="s">
         <v>81</v>
       </c>
       <c r="B42" s="5">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D42" s="5">
-        <v>0</v>
-      </c>
-      <c r="E42" s="5">
-        <v>0</v>
-      </c>
-      <c r="F42" s="5">
-        <v>0</v>
-      </c>
-      <c r="G42" s="5">
-        <v>3</v>
-      </c>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
       <c r="H42" s="6"/>
       <c r="I42" s="6"/>
       <c r="J42" s="6"/>
@@ -2139,25 +3642,17 @@
       <c r="L42" s="6"/>
     </row>
     <row r="43" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="10"/>
+      <c r="A43" s="13"/>
       <c r="B43" s="5">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="D43" s="5">
-        <v>0</v>
-      </c>
-      <c r="E43" s="5">
-        <v>2</v>
-      </c>
-      <c r="F43" s="5">
-        <v>1</v>
-      </c>
-      <c r="G43" s="5">
-        <v>3</v>
-      </c>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
       <c r="H43" s="6"/>
       <c r="I43" s="6"/>
       <c r="J43" s="6"/>
@@ -2167,25 +3662,17 @@
       <c r="L43" s="6"/>
     </row>
     <row r="44" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="10"/>
+      <c r="A44" s="13"/>
       <c r="B44" s="5">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D44" s="5">
-        <v>0</v>
-      </c>
-      <c r="E44" s="5">
-        <v>0</v>
-      </c>
-      <c r="F44" s="5">
-        <v>0</v>
-      </c>
-      <c r="G44" s="5">
-        <v>3</v>
-      </c>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
       <c r="H44" s="6"/>
       <c r="I44" s="6"/>
       <c r="J44" s="6"/>
@@ -2195,25 +3682,17 @@
       <c r="L44" s="6"/>
     </row>
     <row r="45" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="10"/>
+      <c r="A45" s="13"/>
       <c r="B45" s="5">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="D45" s="5">
-        <v>2</v>
-      </c>
-      <c r="E45" s="5">
-        <v>0</v>
-      </c>
-      <c r="F45" s="5">
-        <v>0</v>
-      </c>
-      <c r="G45" s="5">
-        <v>3</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
       <c r="H45" s="6"/>
       <c r="I45" s="6"/>
       <c r="J45" s="6"/>
@@ -2223,25 +3702,17 @@
       <c r="L45" s="6"/>
     </row>
     <row r="46" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="11"/>
+      <c r="A46" s="13"/>
       <c r="B46" s="5">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="D46" s="5">
-        <v>2</v>
-      </c>
-      <c r="E46" s="5">
-        <v>2</v>
-      </c>
-      <c r="F46" s="5">
-        <v>1</v>
-      </c>
-      <c r="G46" s="5">
-        <v>3</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="5"/>
       <c r="H46" s="6"/>
       <c r="I46" s="6"/>
       <c r="J46" s="6"/>
@@ -2250,45 +3721,71 @@
       </c>
       <c r="L46" s="6"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A47" s="8"/>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8" t="s">
+    <row r="47" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="14"/>
+      <c r="B47" s="5">
+        <v>42</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="6"/>
+      <c r="I47" s="6"/>
+      <c r="J47" s="6"/>
+      <c r="K47" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L47" s="6"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A48" s="8"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="D47" s="8">
-        <f>SUM(D5:D46)</f>
-        <v>97</v>
-      </c>
-      <c r="E47" s="8">
-        <f>SUM(E5:E46)</f>
-        <v>62</v>
-      </c>
-      <c r="F47" s="8">
-        <f>SUM(F5:F46)</f>
-        <v>31</v>
-      </c>
-      <c r="G47" s="8">
-        <f>SUM(G5:G46)</f>
-        <v>126</v>
-      </c>
-      <c r="H47" s="8"/>
-      <c r="I47" s="8"/>
-      <c r="J47" s="8"/>
-      <c r="K47" s="8"/>
-      <c r="L47" s="8"/>
+      <c r="D48" s="8">
+        <f>SUM(D5:D47)</f>
+        <v>66</v>
+      </c>
+      <c r="E48" s="8">
+        <f>SUM(E5:E47)</f>
+        <v>34</v>
+      </c>
+      <c r="F48" s="8">
+        <f>SUM(F5:F47)</f>
+        <v>16</v>
+      </c>
+      <c r="G48" s="8">
+        <f>SUM(G5:G47)</f>
+        <v>69</v>
+      </c>
+      <c r="H48" s="8"/>
+      <c r="I48" s="8"/>
+      <c r="J48" s="8"/>
+      <c r="K48" s="8"/>
+      <c r="L48" s="8"/>
+    </row>
+    <row r="53" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D53">
+        <f>COUNT(A5:A47)</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:L47" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="8">
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A42:A47"/>
     <mergeCell ref="A5:A14"/>
-    <mergeCell ref="A15:A21"/>
+    <mergeCell ref="A16:A21"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A24:A30"/>
     <mergeCell ref="A31:A34"/>
     <mergeCell ref="A35:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A42:A46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>

</xml_diff>